<commit_message>
RF SEASONAL: always show real 0s (years 2022/2024/2026 stopped disappearing)
Per sirichai: RF SEASONAL year rows should stay visible even when the
count is genuinely 0, unlike Daily's blank-single-0 rule. Verified there
were 0 real 45RE containers built in 2022/2024/2026 in today's STAYING
stock - not a counting bug, just true zeros that were being hidden.
Applied to both the Excel sheet and the dashboard's RF SEASONAL table.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock Daily 2026-09-22.xlsx
+++ b/Stock Daily 2026-09-22.xlsx
@@ -7343,16 +7343,28 @@
       <c r="A4" s="121" t="n">
         <v>2026</v>
       </c>
-      <c r="B4" s="122" t="n"/>
-      <c r="C4" s="122" t="n"/>
-      <c r="D4" s="122" t="n"/>
+      <c r="B4" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="122" t="n">
+        <v>0</v>
+      </c>
       <c r="E4" s="118" t="n"/>
       <c r="F4" s="122" t="n">
         <v>2026</v>
       </c>
-      <c r="G4" s="122" t="n"/>
-      <c r="H4" s="122" t="n"/>
-      <c r="I4" s="122" t="n"/>
+      <c r="G4" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="122" t="n">
+        <v>0</v>
+      </c>
       <c r="J4" s="120" t="n"/>
       <c r="K4" s="120" t="n"/>
       <c r="L4" s="120" t="n"/>
@@ -7365,8 +7377,12 @@
       <c r="B5" s="123" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="123" t="n"/>
-      <c r="D5" s="123" t="n"/>
+      <c r="C5" s="123" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="123" t="n">
+        <v>0</v>
+      </c>
       <c r="E5" s="118" t="n"/>
       <c r="F5" s="122" t="n">
         <v>2025</v>
@@ -7374,8 +7390,12 @@
       <c r="G5" s="123" t="n">
         <v>7</v>
       </c>
-      <c r="H5" s="123" t="n"/>
-      <c r="I5" s="123" t="n"/>
+      <c r="H5" s="123" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="123" t="n">
+        <v>0</v>
+      </c>
       <c r="J5" s="120" t="n"/>
       <c r="K5" s="120" t="n"/>
       <c r="L5" s="120" t="n"/>
@@ -7385,16 +7405,28 @@
       <c r="A6" s="122" t="n">
         <v>2024</v>
       </c>
-      <c r="B6" s="123" t="n"/>
-      <c r="C6" s="123" t="n"/>
-      <c r="D6" s="123" t="n"/>
+      <c r="B6" s="123" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="123" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="123" t="n">
+        <v>0</v>
+      </c>
       <c r="E6" s="118" t="n"/>
       <c r="F6" s="122" t="n">
         <v>2024</v>
       </c>
-      <c r="G6" s="123" t="n"/>
-      <c r="H6" s="123" t="n"/>
-      <c r="I6" s="123" t="n"/>
+      <c r="G6" s="123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="123" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="123" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="16.15" customHeight="1">
       <c r="A7" s="124" t="n">
@@ -7403,8 +7435,12 @@
       <c r="B7" s="125" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="125" t="n"/>
-      <c r="D7" s="125" t="n"/>
+      <c r="C7" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="125" t="n">
+        <v>0</v>
+      </c>
       <c r="E7" s="111" t="n"/>
       <c r="F7" s="124" t="n">
         <v>2023</v>
@@ -7412,22 +7448,38 @@
       <c r="G7" s="125" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="125" t="n"/>
-      <c r="I7" s="125" t="n"/>
+      <c r="H7" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="16.15" customHeight="1" thickBot="1">
       <c r="A8" s="124" t="n">
         <v>2022</v>
       </c>
-      <c r="B8" s="125" t="n"/>
-      <c r="C8" s="125" t="n"/>
-      <c r="D8" s="125" t="n"/>
+      <c r="B8" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="125" t="n">
+        <v>0</v>
+      </c>
       <c r="F8" s="124" t="n">
         <v>2022</v>
       </c>
-      <c r="G8" s="125" t="n"/>
-      <c r="H8" s="125" t="n"/>
-      <c r="I8" s="125" t="n"/>
+      <c r="G8" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="16.15" customHeight="1" thickTop="1">
       <c r="A9" s="124" t="n">
@@ -7436,16 +7488,24 @@
       <c r="B9" s="125" t="n">
         <v>6</v>
       </c>
-      <c r="C9" s="125" t="n"/>
-      <c r="D9" s="125" t="n"/>
+      <c r="C9" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="125" t="n">
+        <v>0</v>
+      </c>
       <c r="F9" s="124" t="n">
         <v>2021</v>
       </c>
       <c r="G9" s="125" t="n">
         <v>6</v>
       </c>
-      <c r="H9" s="125" t="n"/>
-      <c r="I9" s="125" t="n"/>
+      <c r="H9" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="124" t="n">
@@ -7454,16 +7514,24 @@
       <c r="B10" s="125" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="125" t="n"/>
-      <c r="D10" s="125" t="n"/>
+      <c r="C10" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="125" t="n">
+        <v>0</v>
+      </c>
       <c r="F10" s="124" t="n">
         <v>2020</v>
       </c>
       <c r="G10" s="125" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="125" t="n"/>
-      <c r="I10" s="125" t="n"/>
+      <c r="H10" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="126" t="inlineStr">

</xml_diff>